<commit_message>
modified:   05. PREPROCESSOR & COMPILATION.xlsx
</commit_message>
<xml_diff>
--- a/Kỹ Thuật lập trình/C/00. CheckList.xlsx
+++ b/Kỹ Thuật lập trình/C/00. CheckList.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\WORK\Home\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Document\02.Study\Linux\Kỹ Thuật lập trình\C\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -40,7 +40,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -57,7 +57,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -74,7 +74,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -98,7 +98,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -117,7 +117,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -136,7 +136,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -155,7 +155,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -199,7 +199,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -258,7 +258,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -275,7 +275,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -292,7 +292,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -309,7 +309,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -333,7 +333,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -352,7 +352,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -371,7 +371,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -403,7 +403,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -430,7 +430,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -454,7 +454,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -473,7 +473,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -505,7 +505,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -532,7 +532,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -556,7 +556,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -575,7 +575,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -599,7 +599,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -629,7 +629,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -648,7 +648,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -680,7 +680,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -704,7 +704,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -723,7 +723,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -742,7 +742,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -761,7 +761,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -780,7 +780,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -799,7 +799,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -823,7 +823,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -847,7 +847,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -870,7 +870,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -887,7 +887,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -904,7 +904,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -931,7 +931,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -948,7 +948,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -978,7 +978,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -997,7 +997,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1021,7 +1021,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1040,7 +1040,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1067,7 +1067,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1086,7 +1086,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1105,7 +1105,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1129,7 +1129,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1148,7 +1148,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1186,7 +1186,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1203,7 +1203,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1223,7 +1223,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1250,7 +1250,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1280,7 +1280,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1297,7 +1297,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1327,7 +1327,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1346,7 +1346,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1365,7 +1365,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1389,7 +1389,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1419,7 +1419,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1446,7 +1446,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1463,7 +1463,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1487,7 +1487,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1531,7 +1531,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1548,7 +1548,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1565,7 +1565,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1582,7 +1582,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1636,7 +1636,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1655,7 +1655,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1687,7 +1687,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1704,7 +1704,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1721,7 +1721,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1738,7 +1738,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1780,7 +1780,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1819,7 +1819,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1843,7 +1843,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1866,7 +1866,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1883,7 +1883,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1900,7 +1900,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1945,7 +1945,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1964,7 +1964,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -1983,7 +1983,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2013,7 +2013,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2032,7 +2032,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2059,7 +2059,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2078,7 +2078,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2095,7 +2095,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2112,7 +2112,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2136,7 +2136,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2153,7 +2153,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2180,7 +2180,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2204,7 +2204,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2223,7 +2223,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2253,7 +2253,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2297,7 +2297,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2314,7 +2314,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2331,7 +2331,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2355,7 +2355,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2379,7 +2379,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2409,7 +2409,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2436,7 +2436,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2460,7 +2460,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2487,7 +2487,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2511,7 +2511,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2538,7 +2538,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2557,7 +2557,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2574,7 +2574,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2591,7 +2591,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2608,7 +2608,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2661,7 +2661,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2678,7 +2678,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2705,7 +2705,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2744,7 +2744,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2769,7 +2769,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2786,7 +2786,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2813,7 +2813,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2843,7 +2843,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2870,7 +2870,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2902,7 +2902,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2919,7 +2919,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2936,7 +2936,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2960,7 +2960,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -2979,7 +2979,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3003,7 +3003,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3022,7 +3022,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3041,7 +3041,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3073,7 +3073,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3092,7 +3092,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3116,7 +3116,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3135,7 +3135,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3154,7 +3154,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3173,7 +3173,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3192,7 +3192,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3222,7 +3222,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3246,7 +3246,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3270,7 +3270,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3297,7 +3297,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3317,7 +3317,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3334,7 +3334,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3351,7 +3351,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3375,7 +3375,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3394,7 +3394,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3421,7 +3421,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3445,7 +3445,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3464,7 +3464,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3491,7 +3491,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3510,7 +3510,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3534,7 +3534,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3553,7 +3553,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3583,7 +3583,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3602,7 +3602,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3625,7 +3625,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3649,7 +3649,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3668,7 +3668,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3700,7 +3700,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3731,7 +3731,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3755,7 +3755,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3793,7 +3793,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3810,7 +3810,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3827,7 +3827,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3851,7 +3851,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3886,7 +3886,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3930,7 +3930,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3947,7 +3947,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3964,7 +3964,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -3988,7 +3988,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4012,7 +4012,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4031,7 +4031,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4061,7 +4061,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4080,7 +4080,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4099,7 +4099,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4118,7 +4118,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4148,7 +4148,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4175,7 +4175,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4199,7 +4199,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4219,7 +4219,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4236,7 +4236,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4260,7 +4260,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4279,7 +4279,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4311,7 +4311,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4335,7 +4335,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4354,7 +4354,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4386,7 +4386,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4410,7 +4410,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4434,7 +4434,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4457,7 +4457,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4481,7 +4481,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4505,7 +4505,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4524,7 +4524,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4562,7 +4562,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4579,7 +4579,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4596,7 +4596,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4613,7 +4613,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4637,7 +4637,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4661,7 +4661,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4685,7 +4685,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4704,7 +4704,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4728,7 +4728,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4752,7 +4752,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4771,7 +4771,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4801,7 +4801,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4825,7 +4825,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4844,7 +4844,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4874,7 +4874,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4907,7 +4907,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4924,7 +4924,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4941,7 +4941,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4958,7 +4958,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -4975,7 +4975,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5005,7 +5005,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5029,7 +5029,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5053,7 +5053,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5088,7 +5088,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5112,7 +5112,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5139,7 +5139,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5163,7 +5163,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5182,7 +5182,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5206,7 +5206,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5239,7 +5239,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5256,7 +5256,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5273,7 +5273,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5290,7 +5290,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5307,7 +5307,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5331,7 +5331,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5364,7 +5364,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5414,7 +5414,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5452,7 +5452,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5469,7 +5469,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5493,7 +5493,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5526,7 +5526,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5545,7 +5545,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5571,7 +5571,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5588,7 +5588,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5629,7 +5629,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5658,7 +5658,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5682,7 +5682,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5709,7 +5709,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5728,7 +5728,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5747,7 +5747,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5779,7 +5779,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5796,7 +5796,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5813,7 +5813,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5837,7 +5837,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5861,7 +5861,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5888,7 +5888,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5912,7 +5912,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5939,7 +5939,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5971,7 +5971,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -5988,7 +5988,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6005,7 +6005,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6068,7 +6068,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6092,7 +6092,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6116,7 +6116,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6140,7 +6140,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6172,7 +6172,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6189,7 +6189,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6206,7 +6206,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6259,7 +6259,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6276,7 +6276,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6293,7 +6293,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6349,7 +6349,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6366,7 +6366,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6419,7 +6419,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6436,7 +6436,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6453,7 +6453,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6506,7 +6506,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6523,7 +6523,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6540,7 +6540,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6579,7 +6579,7 @@
       <rPr>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6614,7 +6614,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6631,7 +6631,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6687,7 +6687,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6704,7 +6704,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6721,7 +6721,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6738,7 +6738,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6806,7 +6806,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6823,7 +6823,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6840,7 +6840,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6866,7 +6866,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6922,7 +6922,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6939,7 +6939,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -6995,7 +6995,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7012,7 +7012,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7029,7 +7029,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7082,7 +7082,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7099,7 +7099,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7116,7 +7116,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7169,7 +7169,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7207,7 +7207,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7224,7 +7224,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7241,7 +7241,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7294,7 +7294,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7311,7 +7311,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7328,7 +7328,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7393,7 +7393,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7410,7 +7410,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7463,7 +7463,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7480,7 +7480,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7681,7 +7681,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7698,7 +7698,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7715,7 +7715,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7768,7 +7768,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7785,7 +7785,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7802,7 +7802,7 @@
         <b/>
         <sz val="11"/>
         <color theme="1"/>
-        <rFont val="Calibri"/>
+        <rFont val="Arial"/>
         <family val="2"/>
         <charset val="163"/>
         <scheme val="minor"/>
@@ -7855,7 +7855,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
@@ -7863,7 +7863,7 @@
     <font>
       <sz val="11"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
@@ -7872,7 +7872,7 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
@@ -7881,7 +7881,7 @@
       <b/>
       <sz val="24"/>
       <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
@@ -7890,7 +7890,7 @@
       <b/>
       <sz val="18"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
@@ -7904,7 +7904,7 @@
       <b/>
       <sz val="13.5"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Arial"/>
       <family val="2"/>
       <charset val="163"/>
       <scheme val="minor"/>
@@ -7916,7 +7916,7 @@
       <name val="Arial Unicode MS"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -7926,6 +7926,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -7979,7 +7985,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -8006,6 +8012,11 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -8287,9 +8298,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:AZ350"/>
-  <sheetFormatPr defaultColWidth="3" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="3" defaultRowHeight="14.25"/>
   <sheetData>
-    <row r="2" spans="2:48" ht="31.5">
+    <row r="2" spans="2:48" ht="30">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -8330,7 +8341,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:48">
+    <row r="4" spans="2:48" ht="15">
       <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
@@ -8398,34 +8409,34 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="2:48" ht="15.75" thickBot="1"/>
+    <row r="11" spans="2:48" ht="15" thickBot="1"/>
     <row r="12" spans="2:48" ht="24" thickBot="1">
-      <c r="B12" s="6" t="s">
+      <c r="B12" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
-      <c r="H12" s="7"/>
-      <c r="I12" s="7"/>
-      <c r="J12" s="7"/>
-      <c r="K12" s="7"/>
-      <c r="L12" s="7"/>
-      <c r="M12" s="7"/>
-      <c r="N12" s="7"/>
-      <c r="O12" s="7"/>
-      <c r="P12" s="7"/>
-      <c r="Q12" s="7"/>
-      <c r="R12" s="7"/>
-      <c r="S12" s="7"/>
-      <c r="T12" s="7"/>
-      <c r="U12" s="7"/>
-      <c r="V12" s="7"/>
-      <c r="W12" s="8"/>
-    </row>
-    <row r="14" spans="2:48" ht="18">
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
+      <c r="H12" s="13"/>
+      <c r="I12" s="13"/>
+      <c r="J12" s="13"/>
+      <c r="K12" s="13"/>
+      <c r="L12" s="13"/>
+      <c r="M12" s="13"/>
+      <c r="N12" s="13"/>
+      <c r="O12" s="13"/>
+      <c r="P12" s="13"/>
+      <c r="Q12" s="13"/>
+      <c r="R12" s="13"/>
+      <c r="S12" s="13"/>
+      <c r="T12" s="13"/>
+      <c r="U12" s="13"/>
+      <c r="V12" s="13"/>
+      <c r="W12" s="14"/>
+    </row>
+    <row r="14" spans="2:48" ht="17.25">
       <c r="B14" s="9" t="s">
         <v>21</v>
       </c>
@@ -8439,7 +8450,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="2:48">
+    <row r="15" spans="2:48" ht="15">
       <c r="B15" s="4" t="s">
         <v>25</v>
       </c>
@@ -8519,7 +8530,7 @@
       <c r="AG20" s="4"/>
       <c r="AV20" s="4"/>
     </row>
-    <row r="21" spans="2:48">
+    <row r="21" spans="2:48" ht="15">
       <c r="B21" s="5" t="s">
         <v>47</v>
       </c>
@@ -8531,7 +8542,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="2:48">
+    <row r="22" spans="2:48" ht="15">
       <c r="B22" s="4"/>
       <c r="R22" s="4" t="s">
         <v>50</v>
@@ -8543,7 +8554,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="2:48">
+    <row r="23" spans="2:48" ht="15">
       <c r="B23" s="4" t="s">
         <v>53</v>
       </c>
@@ -8595,7 +8606,7 @@
       <c r="AG26" s="4"/>
       <c r="AV26" s="4"/>
     </row>
-    <row r="27" spans="2:48">
+    <row r="27" spans="2:48" ht="15">
       <c r="B27" s="5" t="s">
         <v>67</v>
       </c>
@@ -8607,7 +8618,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="2:48">
+    <row r="28" spans="2:48" ht="15">
       <c r="B28" s="5" t="s">
         <v>70</v>
       </c>
@@ -8633,7 +8644,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="30" spans="2:48">
+    <row r="30" spans="2:48" ht="15">
       <c r="B30" s="4" t="s">
         <v>77</v>
       </c>
@@ -8667,7 +8678,7 @@
       </c>
       <c r="AG32" s="4"/>
     </row>
-    <row r="33" spans="2:48">
+    <row r="33" spans="2:48" ht="15">
       <c r="B33" s="5" t="s">
         <v>86</v>
       </c>
@@ -8698,33 +8709,33 @@
         <v>92</v>
       </c>
     </row>
-    <row r="38" spans="2:48" ht="15.75" thickBot="1"/>
+    <row r="38" spans="2:48" ht="15" thickBot="1"/>
     <row r="39" spans="2:48" ht="24" thickBot="1">
-      <c r="B39" s="6" t="s">
+      <c r="B39" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="C39" s="7"/>
-      <c r="D39" s="7"/>
-      <c r="E39" s="7"/>
-      <c r="F39" s="7"/>
-      <c r="G39" s="7"/>
-      <c r="H39" s="7"/>
-      <c r="I39" s="7"/>
-      <c r="J39" s="7"/>
-      <c r="K39" s="7"/>
-      <c r="L39" s="7"/>
-      <c r="M39" s="7"/>
-      <c r="N39" s="7"/>
-      <c r="O39" s="7"/>
-      <c r="P39" s="7"/>
-      <c r="Q39" s="7"/>
-      <c r="R39" s="7"/>
-      <c r="S39" s="7"/>
-      <c r="T39" s="7"/>
-      <c r="U39" s="7"/>
-      <c r="V39" s="8"/>
-    </row>
-    <row r="41" spans="2:48" ht="18">
+      <c r="C39" s="13"/>
+      <c r="D39" s="13"/>
+      <c r="E39" s="13"/>
+      <c r="F39" s="13"/>
+      <c r="G39" s="13"/>
+      <c r="H39" s="13"/>
+      <c r="I39" s="13"/>
+      <c r="J39" s="13"/>
+      <c r="K39" s="13"/>
+      <c r="L39" s="13"/>
+      <c r="M39" s="13"/>
+      <c r="N39" s="13"/>
+      <c r="O39" s="13"/>
+      <c r="P39" s="13"/>
+      <c r="Q39" s="13"/>
+      <c r="R39" s="13"/>
+      <c r="S39" s="13"/>
+      <c r="T39" s="13"/>
+      <c r="U39" s="13"/>
+      <c r="V39" s="14"/>
+    </row>
+    <row r="41" spans="2:48" ht="17.25">
       <c r="B41" s="9" t="s">
         <v>94</v>
       </c>
@@ -8738,7 +8749,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="42" spans="2:48">
+    <row r="42" spans="2:48" ht="15">
       <c r="B42" s="4" t="s">
         <v>98</v>
       </c>
@@ -8814,7 +8825,7 @@
       <c r="AG47" s="4"/>
       <c r="AV47" s="4"/>
     </row>
-    <row r="48" spans="2:48">
+    <row r="48" spans="2:48" ht="15">
       <c r="B48" s="4" t="s">
         <v>118</v>
       </c>
@@ -8889,7 +8900,7 @@
       <c r="R53" s="4"/>
       <c r="AG53" s="4"/>
     </row>
-    <row r="54" spans="2:48">
+    <row r="54" spans="2:48" ht="15">
       <c r="B54" s="4" t="s">
         <v>138</v>
       </c>
@@ -8951,7 +8962,7 @@
       </c>
       <c r="AG59" s="4"/>
     </row>
-    <row r="60" spans="2:48">
+    <row r="60" spans="2:48" ht="15">
       <c r="B60" s="4" t="s">
         <v>154</v>
       </c>
@@ -8960,7 +8971,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="61" spans="2:48">
+    <row r="61" spans="2:48" ht="15">
       <c r="B61" s="5" t="s">
         <v>156</v>
       </c>
@@ -9009,27 +9020,27 @@
         <v>168</v>
       </c>
     </row>
-    <row r="66" spans="2:33" ht="15.75" thickBot="1"/>
+    <row r="66" spans="2:33" ht="15" thickBot="1"/>
     <row r="67" spans="2:33" ht="24" thickBot="1">
-      <c r="B67" s="6" t="s">
+      <c r="B67" s="12" t="s">
         <v>169</v>
       </c>
-      <c r="C67" s="7"/>
-      <c r="D67" s="7"/>
-      <c r="E67" s="7"/>
-      <c r="F67" s="7"/>
-      <c r="G67" s="7"/>
-      <c r="H67" s="7"/>
-      <c r="I67" s="7"/>
-      <c r="J67" s="7"/>
-      <c r="K67" s="7"/>
-      <c r="L67" s="7"/>
-      <c r="M67" s="7"/>
-      <c r="N67" s="7"/>
-      <c r="O67" s="7"/>
-      <c r="P67" s="8"/>
-    </row>
-    <row r="68" spans="2:33" ht="18">
+      <c r="C67" s="13"/>
+      <c r="D67" s="13"/>
+      <c r="E67" s="13"/>
+      <c r="F67" s="13"/>
+      <c r="G67" s="13"/>
+      <c r="H67" s="13"/>
+      <c r="I67" s="13"/>
+      <c r="J67" s="13"/>
+      <c r="K67" s="13"/>
+      <c r="L67" s="13"/>
+      <c r="M67" s="13"/>
+      <c r="N67" s="13"/>
+      <c r="O67" s="13"/>
+      <c r="P67" s="14"/>
+    </row>
+    <row r="68" spans="2:33" ht="17.25">
       <c r="B68" s="9" t="s">
         <v>170</v>
       </c>
@@ -9040,7 +9051,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="69" spans="2:33">
+    <row r="69" spans="2:33" ht="15">
       <c r="B69" s="4" t="s">
         <v>173</v>
       </c>
@@ -9102,7 +9113,7 @@
       <c r="R74" s="4"/>
       <c r="AG74" s="4"/>
     </row>
-    <row r="75" spans="2:33">
+    <row r="75" spans="2:33" ht="15">
       <c r="B75" s="4"/>
       <c r="R75" s="4" t="s">
         <v>189</v>
@@ -9111,7 +9122,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="76" spans="2:33">
+    <row r="76" spans="2:33" ht="15">
       <c r="B76" s="4" t="s">
         <v>191</v>
       </c>
@@ -9161,13 +9172,13 @@
       </c>
       <c r="R80" s="4"/>
     </row>
-    <row r="81" spans="2:32">
+    <row r="81" spans="2:32" ht="15">
       <c r="B81" s="4"/>
       <c r="R81" s="4" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="82" spans="2:32">
+    <row r="82" spans="2:32" ht="15">
       <c r="B82" s="4" t="s">
         <v>205</v>
       </c>
@@ -9205,13 +9216,13 @@
       </c>
       <c r="R86" s="4"/>
     </row>
-    <row r="87" spans="2:32">
+    <row r="87" spans="2:32" ht="15">
       <c r="B87" s="4"/>
       <c r="R87" s="4" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="88" spans="2:32">
+    <row r="88" spans="2:32" ht="15">
       <c r="B88" s="4" t="s">
         <v>215</v>
       </c>
@@ -9248,32 +9259,32 @@
         <v>223</v>
       </c>
     </row>
-    <row r="93" spans="2:32" ht="15.75" thickBot="1"/>
+    <row r="93" spans="2:32" ht="15" thickBot="1"/>
     <row r="94" spans="2:32" ht="24" thickBot="1">
-      <c r="B94" s="6" t="s">
+      <c r="B94" s="12" t="s">
         <v>224</v>
       </c>
-      <c r="C94" s="7"/>
-      <c r="D94" s="7"/>
-      <c r="E94" s="7"/>
-      <c r="F94" s="7"/>
-      <c r="G94" s="7"/>
-      <c r="H94" s="7"/>
-      <c r="I94" s="7"/>
-      <c r="J94" s="7"/>
-      <c r="K94" s="7"/>
-      <c r="L94" s="7"/>
-      <c r="M94" s="7"/>
-      <c r="N94" s="7"/>
-      <c r="O94" s="7"/>
-      <c r="P94" s="7"/>
-      <c r="Q94" s="7"/>
-      <c r="R94" s="7"/>
-      <c r="S94" s="7"/>
-      <c r="T94" s="7"/>
-      <c r="U94" s="8"/>
-    </row>
-    <row r="95" spans="2:32" ht="18">
+      <c r="C94" s="13"/>
+      <c r="D94" s="13"/>
+      <c r="E94" s="13"/>
+      <c r="F94" s="13"/>
+      <c r="G94" s="13"/>
+      <c r="H94" s="13"/>
+      <c r="I94" s="13"/>
+      <c r="J94" s="13"/>
+      <c r="K94" s="13"/>
+      <c r="L94" s="13"/>
+      <c r="M94" s="13"/>
+      <c r="N94" s="13"/>
+      <c r="O94" s="13"/>
+      <c r="P94" s="13"/>
+      <c r="Q94" s="13"/>
+      <c r="R94" s="13"/>
+      <c r="S94" s="13"/>
+      <c r="T94" s="13"/>
+      <c r="U94" s="14"/>
+    </row>
+    <row r="95" spans="2:32" ht="17.25">
       <c r="B95" s="9" t="s">
         <v>225</v>
       </c>
@@ -9284,7 +9295,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="96" spans="2:32">
+    <row r="96" spans="2:32" ht="15">
       <c r="B96" s="4" t="s">
         <v>228</v>
       </c>
@@ -9344,7 +9355,7 @@
       <c r="R101" s="4"/>
       <c r="AF101" s="4"/>
     </row>
-    <row r="102" spans="2:32">
+    <row r="102" spans="2:32" ht="15">
       <c r="B102" s="4" t="s">
         <v>243</v>
       </c>
@@ -9402,7 +9413,7 @@
     <row r="107" spans="2:32">
       <c r="B107" s="4"/>
     </row>
-    <row r="108" spans="2:32">
+    <row r="108" spans="2:32" ht="15">
       <c r="B108" s="4" t="s">
         <v>258</v>
       </c>
@@ -9430,7 +9441,7 @@
     <row r="113" spans="2:33">
       <c r="B113" s="4"/>
     </row>
-    <row r="114" spans="2:33">
+    <row r="114" spans="2:33" ht="15">
       <c r="B114" s="4" t="s">
         <v>263</v>
       </c>
@@ -9455,31 +9466,31 @@
         <v>267</v>
       </c>
     </row>
-    <row r="119" spans="2:33" ht="15.75" thickBot="1"/>
+    <row r="119" spans="2:33" ht="15" thickBot="1"/>
     <row r="120" spans="2:33" ht="24" thickBot="1">
-      <c r="B120" s="6" t="s">
+      <c r="B120" s="12" t="s">
         <v>268</v>
       </c>
-      <c r="C120" s="7"/>
-      <c r="D120" s="7"/>
-      <c r="E120" s="7"/>
-      <c r="F120" s="7"/>
-      <c r="G120" s="7"/>
-      <c r="H120" s="7"/>
-      <c r="I120" s="7"/>
-      <c r="J120" s="7"/>
-      <c r="K120" s="7"/>
-      <c r="L120" s="7"/>
-      <c r="M120" s="7"/>
-      <c r="N120" s="7"/>
-      <c r="O120" s="7"/>
-      <c r="P120" s="7"/>
-      <c r="Q120" s="7"/>
-      <c r="R120" s="7"/>
-      <c r="S120" s="7"/>
-      <c r="T120" s="8"/>
-    </row>
-    <row r="121" spans="2:33" ht="18">
+      <c r="C120" s="13"/>
+      <c r="D120" s="13"/>
+      <c r="E120" s="13"/>
+      <c r="F120" s="13"/>
+      <c r="G120" s="13"/>
+      <c r="H120" s="13"/>
+      <c r="I120" s="13"/>
+      <c r="J120" s="13"/>
+      <c r="K120" s="13"/>
+      <c r="L120" s="13"/>
+      <c r="M120" s="13"/>
+      <c r="N120" s="13"/>
+      <c r="O120" s="13"/>
+      <c r="P120" s="13"/>
+      <c r="Q120" s="13"/>
+      <c r="R120" s="13"/>
+      <c r="S120" s="13"/>
+      <c r="T120" s="14"/>
+    </row>
+    <row r="121" spans="2:33" ht="17.25">
       <c r="B121" s="9" t="s">
         <v>269</v>
       </c>
@@ -9490,7 +9501,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="122" spans="2:33">
+    <row r="122" spans="2:33" ht="15">
       <c r="B122" s="4" t="s">
         <v>272</v>
       </c>
@@ -9550,7 +9561,7 @@
       <c r="R127" s="4"/>
       <c r="AG127" s="4"/>
     </row>
-    <row r="128" spans="2:33">
+    <row r="128" spans="2:33" ht="15">
       <c r="B128" s="4" t="s">
         <v>287</v>
       </c>
@@ -9609,7 +9620,7 @@
       <c r="B133" s="4"/>
       <c r="R133" s="4"/>
     </row>
-    <row r="134" spans="2:33">
+    <row r="134" spans="2:33" ht="15">
       <c r="B134" s="4" t="s">
         <v>302</v>
       </c>
@@ -9652,7 +9663,7 @@
     <row r="139" spans="2:33">
       <c r="B139" s="4"/>
     </row>
-    <row r="140" spans="2:33">
+    <row r="140" spans="2:33" ht="15">
       <c r="B140" s="4" t="s">
         <v>312</v>
       </c>
@@ -9704,7 +9715,7 @@
       <c r="W146" s="11"/>
       <c r="X146" s="11"/>
     </row>
-    <row r="147" spans="2:48" ht="18">
+    <row r="147" spans="2:48" ht="17.25">
       <c r="B147" s="9" t="s">
         <v>318</v>
       </c>
@@ -9718,7 +9729,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="148" spans="2:48">
+    <row r="148" spans="2:48" ht="15">
       <c r="B148" s="4" t="s">
         <v>322</v>
       </c>
@@ -9794,7 +9805,7 @@
       <c r="AG153" s="4"/>
       <c r="AV153" s="4"/>
     </row>
-    <row r="154" spans="2:48">
+    <row r="154" spans="2:48" ht="15">
       <c r="B154" s="4" t="s">
         <v>342</v>
       </c>
@@ -9870,7 +9881,7 @@
       <c r="AG159" s="4"/>
       <c r="AV159" s="4"/>
     </row>
-    <row r="160" spans="2:48">
+    <row r="160" spans="2:48" ht="15">
       <c r="B160" s="4" t="s">
         <v>362</v>
       </c>
@@ -9943,7 +9954,7 @@
     <row r="165" spans="2:48">
       <c r="R165" s="4"/>
     </row>
-    <row r="166" spans="2:48">
+    <row r="166" spans="2:48" ht="15">
       <c r="R166" s="4" t="s">
         <v>382</v>
       </c>
@@ -9968,7 +9979,7 @@
         <v>386</v>
       </c>
     </row>
-    <row r="172" spans="2:48" ht="15.75" thickBot="1"/>
+    <row r="172" spans="2:48" ht="15" thickBot="1"/>
     <row r="173" spans="2:48" ht="24" thickBot="1">
       <c r="B173" s="6" t="s">
         <v>387</v>
@@ -9988,7 +9999,7 @@
       <c r="O173" s="7"/>
       <c r="P173" s="8"/>
     </row>
-    <row r="174" spans="2:48" ht="18">
+    <row r="174" spans="2:48" ht="17.25">
       <c r="B174" s="9" t="s">
         <v>388</v>
       </c>
@@ -9996,7 +10007,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="175" spans="2:48">
+    <row r="175" spans="2:48" ht="15">
       <c r="B175" s="4" t="s">
         <v>390</v>
       </c>
@@ -10040,7 +10051,7 @@
       <c r="B180" s="4"/>
       <c r="R180" s="4"/>
     </row>
-    <row r="181" spans="2:18">
+    <row r="181" spans="2:18" ht="15">
       <c r="B181" s="4" t="s">
         <v>400</v>
       </c>
@@ -10083,7 +10094,7 @@
     <row r="186" spans="2:18">
       <c r="B186" s="4"/>
     </row>
-    <row r="187" spans="2:18">
+    <row r="187" spans="2:18" ht="15">
       <c r="B187" s="4" t="s">
         <v>410</v>
       </c>
@@ -10111,7 +10122,7 @@
     <row r="192" spans="2:18">
       <c r="B192" s="4"/>
     </row>
-    <row r="193" spans="2:29">
+    <row r="193" spans="2:29" ht="15">
       <c r="B193" s="4" t="s">
         <v>415</v>
       </c>
@@ -10136,7 +10147,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="198" spans="2:29" ht="15.75" thickBot="1"/>
+    <row r="198" spans="2:29" ht="15" thickBot="1"/>
     <row r="199" spans="2:29" ht="24" thickBot="1">
       <c r="B199" s="6" t="s">
         <v>420</v>
@@ -10155,7 +10166,7 @@
       <c r="N199" s="7"/>
       <c r="O199" s="8"/>
     </row>
-    <row r="200" spans="2:29" ht="18">
+    <row r="200" spans="2:29" ht="17.25">
       <c r="B200" s="9" t="s">
         <v>421</v>
       </c>
@@ -10166,7 +10177,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="201" spans="2:29">
+    <row r="201" spans="2:29" ht="15">
       <c r="B201" s="4" t="s">
         <v>424</v>
       </c>
@@ -10226,7 +10237,7 @@
       <c r="R206" s="4"/>
       <c r="AC206" s="4"/>
     </row>
-    <row r="207" spans="2:29">
+    <row r="207" spans="2:29" ht="15">
       <c r="B207" s="4" t="s">
         <v>439</v>
       </c>
@@ -10284,7 +10295,7 @@
     <row r="212" spans="2:33">
       <c r="B212" s="4"/>
     </row>
-    <row r="213" spans="2:33">
+    <row r="213" spans="2:33" ht="15">
       <c r="B213" s="4" t="s">
         <v>454</v>
       </c>
@@ -10309,7 +10320,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="219" spans="2:33" ht="15.75" thickBot="1"/>
+    <row r="219" spans="2:33" ht="15" thickBot="1"/>
     <row r="220" spans="2:33" ht="24" thickBot="1">
       <c r="B220" s="6" t="s">
         <v>459</v>
@@ -10329,7 +10340,7 @@
       <c r="O220" s="7"/>
       <c r="P220" s="8"/>
     </row>
-    <row r="221" spans="2:33" ht="18">
+    <row r="221" spans="2:33" ht="17.25">
       <c r="B221" s="9" t="s">
         <v>460</v>
       </c>
@@ -10340,7 +10351,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="222" spans="2:33">
+    <row r="222" spans="2:33" ht="15">
       <c r="B222" s="4" t="s">
         <v>463</v>
       </c>
@@ -10400,7 +10411,7 @@
       <c r="P227" s="4"/>
       <c r="AG227" s="4"/>
     </row>
-    <row r="228" spans="2:33">
+    <row r="228" spans="2:33" ht="15">
       <c r="B228" s="4" t="s">
         <v>478</v>
       </c>
@@ -10461,13 +10472,13 @@
       </c>
       <c r="P233" s="4"/>
     </row>
-    <row r="234" spans="2:33">
+    <row r="234" spans="2:33" ht="15">
       <c r="B234" s="4"/>
       <c r="P234" s="4" t="s">
         <v>494</v>
       </c>
     </row>
-    <row r="235" spans="2:33">
+    <row r="235" spans="2:33" ht="15">
       <c r="B235" s="4" t="s">
         <v>495</v>
       </c>
@@ -10504,7 +10515,7 @@
         <v>503</v>
       </c>
     </row>
-    <row r="240" spans="2:33" ht="15.75" thickBot="1"/>
+    <row r="240" spans="2:33" ht="15" thickBot="1"/>
     <row r="241" spans="2:33" ht="24" thickBot="1">
       <c r="B241" s="6" t="s">
         <v>504</v>
@@ -10523,7 +10534,7 @@
       <c r="N241" s="7"/>
       <c r="O241" s="8"/>
     </row>
-    <row r="242" spans="2:33" ht="18">
+    <row r="242" spans="2:33" ht="17.25">
       <c r="B242" s="9" t="s">
         <v>505</v>
       </c>
@@ -10534,7 +10545,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="243" spans="2:33">
+    <row r="243" spans="2:33" ht="15">
       <c r="B243" s="4" t="s">
         <v>508</v>
       </c>
@@ -10594,7 +10605,7 @@
       <c r="P248" s="4"/>
       <c r="AG248" s="4"/>
     </row>
-    <row r="249" spans="2:33">
+    <row r="249" spans="2:33" ht="15">
       <c r="B249" s="4" t="s">
         <v>523</v>
       </c>
@@ -10653,7 +10664,7 @@
       <c r="B254" s="4"/>
       <c r="P254" s="4"/>
     </row>
-    <row r="255" spans="2:33">
+    <row r="255" spans="2:33" ht="15">
       <c r="B255" s="4" t="s">
         <v>538</v>
       </c>
@@ -10693,7 +10704,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="260" spans="2:41" ht="15.75" thickBot="1"/>
+    <row r="260" spans="2:41" ht="15" thickBot="1"/>
     <row r="261" spans="2:41" ht="24" thickBot="1">
       <c r="B261" s="6" t="s">
         <v>548</v>
@@ -10718,7 +10729,7 @@
       <c r="T261" s="7"/>
       <c r="U261" s="8"/>
     </row>
-    <row r="262" spans="2:41" ht="18">
+    <row r="262" spans="2:41" ht="17.25">
       <c r="B262" s="9" t="s">
         <v>549</v>
       </c>
@@ -10732,7 +10743,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="263" spans="2:41">
+    <row r="263" spans="2:41" ht="15">
       <c r="B263" s="4" t="s">
         <v>553</v>
       </c>
@@ -10810,7 +10821,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="269" spans="2:41">
+    <row r="269" spans="2:41" ht="15">
       <c r="B269" s="4" t="s">
         <v>574</v>
       </c>
@@ -10822,7 +10833,7 @@
       </c>
       <c r="AO269" s="4"/>
     </row>
-    <row r="270" spans="2:41">
+    <row r="270" spans="2:41" ht="15">
       <c r="B270" s="5" t="s">
         <v>577</v>
       </c>
@@ -10885,7 +10896,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="275" spans="2:41">
+    <row r="275" spans="2:41" ht="15">
       <c r="B275" s="4" t="s">
         <v>594</v>
       </c>
@@ -10930,7 +10941,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="281" spans="2:41" ht="15.75" thickBot="1"/>
+    <row r="281" spans="2:41" ht="15" thickBot="1"/>
     <row r="282" spans="2:41" ht="24" thickBot="1">
       <c r="B282" s="6" t="s">
         <v>605</v>
@@ -10952,7 +10963,7 @@
       <c r="Q282" s="7"/>
       <c r="R282" s="8"/>
     </row>
-    <row r="283" spans="2:41" ht="18">
+    <row r="283" spans="2:41" ht="17.25">
       <c r="B283" s="9" t="s">
         <v>606</v>
       </c>
@@ -10963,7 +10974,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="284" spans="2:41">
+    <row r="284" spans="2:41" ht="15">
       <c r="B284" s="4" t="s">
         <v>609</v>
       </c>
@@ -11023,7 +11034,7 @@
       <c r="Q289" s="4"/>
       <c r="AC289" s="4"/>
     </row>
-    <row r="290" spans="2:29">
+    <row r="290" spans="2:29" ht="15">
       <c r="B290" s="4" t="s">
         <v>624</v>
       </c>
@@ -11081,7 +11092,7 @@
     <row r="295" spans="2:29">
       <c r="B295" s="4"/>
     </row>
-    <row r="296" spans="2:29">
+    <row r="296" spans="2:29" ht="15">
       <c r="B296" s="4" t="s">
         <v>639</v>
       </c>
@@ -11106,7 +11117,7 @@
         <v>642</v>
       </c>
     </row>
-    <row r="301" spans="2:29" ht="15.75" thickBot="1"/>
+    <row r="301" spans="2:29" ht="15" thickBot="1"/>
     <row r="302" spans="2:29" ht="24" thickBot="1">
       <c r="B302" s="6" t="s">
         <v>643</v>
@@ -11132,7 +11143,7 @@
       <c r="U302" s="7"/>
       <c r="V302" s="8"/>
     </row>
-    <row r="303" spans="2:29" ht="18">
+    <row r="303" spans="2:29" ht="17.25">
       <c r="B303" s="9" t="s">
         <v>644</v>
       </c>
@@ -11143,7 +11154,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="304" spans="2:29">
+    <row r="304" spans="2:29" ht="15">
       <c r="B304" s="4" t="s">
         <v>647</v>
       </c>
@@ -11203,7 +11214,7 @@
       <c r="P309" s="4"/>
       <c r="AC309" s="4"/>
     </row>
-    <row r="310" spans="2:29">
+    <row r="310" spans="2:29" ht="15">
       <c r="B310" s="4" t="s">
         <v>662</v>
       </c>
@@ -11258,7 +11269,7 @@
         <v>676</v>
       </c>
     </row>
-    <row r="315" spans="2:29" ht="15.75" thickBot="1"/>
+    <row r="315" spans="2:29" ht="15" thickBot="1"/>
     <row r="316" spans="2:29" ht="24" thickBot="1">
       <c r="B316" s="6" t="s">
         <v>677</v>
@@ -11281,7 +11292,7 @@
       <c r="R316" s="7"/>
       <c r="S316" s="8"/>
     </row>
-    <row r="317" spans="2:29" ht="18">
+    <row r="317" spans="2:29" ht="17.25">
       <c r="B317" s="9" t="s">
         <v>678</v>
       </c>
@@ -11292,7 +11303,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="318" spans="2:29">
+    <row r="318" spans="2:29" ht="15">
       <c r="B318" s="4" t="s">
         <v>681</v>
       </c>
@@ -11351,7 +11362,7 @@
       <c r="B323" s="4"/>
       <c r="P323" s="4"/>
     </row>
-    <row r="324" spans="2:52">
+    <row r="324" spans="2:52" ht="15">
       <c r="B324" s="4" t="s">
         <v>695</v>
       </c>
@@ -11391,7 +11402,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="329" spans="2:52" ht="15.75" thickBot="1"/>
+    <row r="329" spans="2:52" ht="15" thickBot="1"/>
     <row r="330" spans="2:52" ht="24" thickBot="1">
       <c r="B330" s="6" t="s">
         <v>705</v>
@@ -11409,7 +11420,7 @@
       <c r="M330" s="7"/>
       <c r="N330" s="8"/>
     </row>
-    <row r="331" spans="2:52" ht="18">
+    <row r="331" spans="2:52" ht="17.25">
       <c r="B331" s="9" t="s">
         <v>706</v>
       </c>
@@ -11511,7 +11522,7 @@
         <v>735</v>
       </c>
     </row>
-    <row r="337" spans="2:29" ht="15.75" thickBot="1"/>
+    <row r="337" spans="2:29" ht="15" thickBot="1"/>
     <row r="338" spans="2:29" ht="24" thickBot="1">
       <c r="B338" s="6" t="s">
         <v>736</v>
@@ -11530,7 +11541,7 @@
       <c r="N338" s="7"/>
       <c r="O338" s="8"/>
     </row>
-    <row r="339" spans="2:29" ht="18">
+    <row r="339" spans="2:29" ht="17.25">
       <c r="B339" s="9" t="s">
         <v>737</v>
       </c>
@@ -11541,7 +11552,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="340" spans="2:29">
+    <row r="340" spans="2:29" ht="15">
       <c r="B340" s="4" t="s">
         <v>740</v>
       </c>
@@ -11601,7 +11612,7 @@
       <c r="P345" s="4"/>
       <c r="AC345" s="4"/>
     </row>
-    <row r="346" spans="2:29">
+    <row r="346" spans="2:29" ht="15">
       <c r="B346" s="4" t="s">
         <v>755</v>
       </c>

</xml_diff>

<commit_message>
[200~ modified:   00. CheckList.xlsx
</commit_message>
<xml_diff>
--- a/Kỹ Thuật lập trình/C/00. CheckList.xlsx
+++ b/Kỹ Thuật lập trình/C/00. CheckList.xlsx
@@ -8298,7 +8298,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B2:AZ350"/>
-  <sheetFormatPr defaultColWidth="3" defaultRowHeight="14.25"/>
+  <sheetFormatPr defaultColWidth="3" defaultRowHeight="13.8"/>
   <sheetData>
     <row r="2" spans="2:48" ht="30">
       <c r="B2" s="1" t="s">
@@ -8336,12 +8336,12 @@
       <c r="AF2" s="2"/>
       <c r="AG2" s="2"/>
     </row>
-    <row r="3" spans="2:48" ht="23.25">
+    <row r="3" spans="2:48" ht="22.8">
       <c r="B3" s="3" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="2:48" ht="15">
+    <row r="4" spans="2:48">
       <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
@@ -8409,8 +8409,8 @@
         <v>19</v>
       </c>
     </row>
-    <row r="11" spans="2:48" ht="15" thickBot="1"/>
-    <row r="12" spans="2:48" ht="24" thickBot="1">
+    <row r="11" spans="2:48" ht="14.4" thickBot="1"/>
+    <row r="12" spans="2:48" ht="23.4" thickBot="1">
       <c r="B12" s="10" t="s">
         <v>20</v>
       </c>
@@ -8436,7 +8436,7 @@
       <c r="V12" s="11"/>
       <c r="W12" s="12"/>
     </row>
-    <row r="14" spans="2:48" ht="17.25">
+    <row r="14" spans="2:48" ht="17.399999999999999">
       <c r="B14" s="9" t="s">
         <v>21</v>
       </c>
@@ -8450,7 +8450,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="2:48" ht="15">
+    <row r="15" spans="2:48">
       <c r="B15" s="4" t="s">
         <v>25</v>
       </c>
@@ -8530,7 +8530,7 @@
       <c r="AG20" s="4"/>
       <c r="AV20" s="4"/>
     </row>
-    <row r="21" spans="2:48" ht="15">
+    <row r="21" spans="2:48">
       <c r="B21" s="5" t="s">
         <v>47</v>
       </c>
@@ -8542,7 +8542,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="2:48" ht="15">
+    <row r="22" spans="2:48">
       <c r="B22" s="4"/>
       <c r="R22" s="4" t="s">
         <v>50</v>
@@ -8554,7 +8554,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="23" spans="2:48" ht="15">
+    <row r="23" spans="2:48">
       <c r="B23" s="4" t="s">
         <v>53</v>
       </c>
@@ -8606,7 +8606,7 @@
       <c r="AG26" s="4"/>
       <c r="AV26" s="4"/>
     </row>
-    <row r="27" spans="2:48" ht="15">
+    <row r="27" spans="2:48">
       <c r="B27" s="5" t="s">
         <v>67</v>
       </c>
@@ -8618,7 +8618,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="2:48" ht="15">
+    <row r="28" spans="2:48">
       <c r="B28" s="5" t="s">
         <v>70</v>
       </c>
@@ -8644,7 +8644,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="30" spans="2:48" ht="15">
+    <row r="30" spans="2:48">
       <c r="B30" s="4" t="s">
         <v>77</v>
       </c>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="AG32" s="4"/>
     </row>
-    <row r="33" spans="2:48" ht="15">
+    <row r="33" spans="2:48">
       <c r="B33" s="5" t="s">
         <v>86</v>
       </c>
@@ -8709,8 +8709,8 @@
         <v>92</v>
       </c>
     </row>
-    <row r="38" spans="2:48" ht="15" thickBot="1"/>
-    <row r="39" spans="2:48" ht="24" thickBot="1">
+    <row r="38" spans="2:48" ht="14.4" thickBot="1"/>
+    <row r="39" spans="2:48" ht="23.4" thickBot="1">
       <c r="B39" s="10" t="s">
         <v>93</v>
       </c>
@@ -8735,7 +8735,7 @@
       <c r="U39" s="11"/>
       <c r="V39" s="12"/>
     </row>
-    <row r="41" spans="2:48" ht="17.25">
+    <row r="41" spans="2:48" ht="17.399999999999999">
       <c r="B41" s="9" t="s">
         <v>94</v>
       </c>
@@ -8749,7 +8749,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="42" spans="2:48" ht="15">
+    <row r="42" spans="2:48">
       <c r="B42" s="4" t="s">
         <v>98</v>
       </c>
@@ -8825,7 +8825,7 @@
       <c r="AG47" s="4"/>
       <c r="AV47" s="4"/>
     </row>
-    <row r="48" spans="2:48" ht="15">
+    <row r="48" spans="2:48">
       <c r="B48" s="4" t="s">
         <v>118</v>
       </c>
@@ -8900,7 +8900,7 @@
       <c r="R53" s="4"/>
       <c r="AG53" s="4"/>
     </row>
-    <row r="54" spans="2:48" ht="15">
+    <row r="54" spans="2:48">
       <c r="B54" s="4" t="s">
         <v>138</v>
       </c>
@@ -8962,7 +8962,7 @@
       </c>
       <c r="AG59" s="4"/>
     </row>
-    <row r="60" spans="2:48" ht="15">
+    <row r="60" spans="2:48">
       <c r="B60" s="4" t="s">
         <v>154</v>
       </c>
@@ -8971,7 +8971,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="61" spans="2:48" ht="15">
+    <row r="61" spans="2:48">
       <c r="B61" s="5" t="s">
         <v>156</v>
       </c>
@@ -9020,8 +9020,8 @@
         <v>168</v>
       </c>
     </row>
-    <row r="66" spans="2:33" ht="15" thickBot="1"/>
-    <row r="67" spans="2:33" ht="24" thickBot="1">
+    <row r="66" spans="2:33" ht="14.4" thickBot="1"/>
+    <row r="67" spans="2:33" ht="23.4" thickBot="1">
       <c r="B67" s="10" t="s">
         <v>169</v>
       </c>
@@ -9040,7 +9040,7 @@
       <c r="O67" s="11"/>
       <c r="P67" s="12"/>
     </row>
-    <row r="68" spans="2:33" ht="17.25">
+    <row r="68" spans="2:33" ht="17.399999999999999">
       <c r="B68" s="9" t="s">
         <v>170</v>
       </c>
@@ -9051,7 +9051,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="69" spans="2:33" ht="15">
+    <row r="69" spans="2:33">
       <c r="B69" s="4" t="s">
         <v>173</v>
       </c>
@@ -9113,7 +9113,7 @@
       <c r="R74" s="4"/>
       <c r="AG74" s="4"/>
     </row>
-    <row r="75" spans="2:33" ht="15">
+    <row r="75" spans="2:33">
       <c r="B75" s="4"/>
       <c r="R75" s="4" t="s">
         <v>189</v>
@@ -9122,7 +9122,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="76" spans="2:33" ht="15">
+    <row r="76" spans="2:33">
       <c r="B76" s="4" t="s">
         <v>191</v>
       </c>
@@ -9172,13 +9172,13 @@
       </c>
       <c r="R80" s="4"/>
     </row>
-    <row r="81" spans="2:32" ht="15">
+    <row r="81" spans="2:32">
       <c r="B81" s="4"/>
       <c r="R81" s="4" t="s">
         <v>204</v>
       </c>
     </row>
-    <row r="82" spans="2:32" ht="15">
+    <row r="82" spans="2:32">
       <c r="B82" s="4" t="s">
         <v>205</v>
       </c>
@@ -9216,13 +9216,13 @@
       </c>
       <c r="R86" s="4"/>
     </row>
-    <row r="87" spans="2:32" ht="15">
+    <row r="87" spans="2:32">
       <c r="B87" s="4"/>
       <c r="R87" s="4" t="s">
         <v>214</v>
       </c>
     </row>
-    <row r="88" spans="2:32" ht="15">
+    <row r="88" spans="2:32">
       <c r="B88" s="4" t="s">
         <v>215</v>
       </c>
@@ -9259,8 +9259,8 @@
         <v>223</v>
       </c>
     </row>
-    <row r="93" spans="2:32" ht="15" thickBot="1"/>
-    <row r="94" spans="2:32" ht="24" thickBot="1">
+    <row r="93" spans="2:32" ht="14.4" thickBot="1"/>
+    <row r="94" spans="2:32" ht="23.4" thickBot="1">
       <c r="B94" s="10" t="s">
         <v>224</v>
       </c>
@@ -9284,7 +9284,7 @@
       <c r="T94" s="11"/>
       <c r="U94" s="12"/>
     </row>
-    <row r="95" spans="2:32" ht="17.25">
+    <row r="95" spans="2:32" ht="17.399999999999999">
       <c r="B95" s="9" t="s">
         <v>225</v>
       </c>
@@ -9295,7 +9295,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="96" spans="2:32" ht="15">
+    <row r="96" spans="2:32">
       <c r="B96" s="4" t="s">
         <v>228</v>
       </c>
@@ -9355,7 +9355,7 @@
       <c r="R101" s="4"/>
       <c r="AF101" s="4"/>
     </row>
-    <row r="102" spans="2:32" ht="15">
+    <row r="102" spans="2:32">
       <c r="B102" s="4" t="s">
         <v>243</v>
       </c>
@@ -9413,7 +9413,7 @@
     <row r="107" spans="2:32">
       <c r="B107" s="4"/>
     </row>
-    <row r="108" spans="2:32" ht="15">
+    <row r="108" spans="2:32">
       <c r="B108" s="4" t="s">
         <v>258</v>
       </c>
@@ -9441,7 +9441,7 @@
     <row r="113" spans="2:33">
       <c r="B113" s="4"/>
     </row>
-    <row r="114" spans="2:33" ht="15">
+    <row r="114" spans="2:33">
       <c r="B114" s="4" t="s">
         <v>263</v>
       </c>
@@ -9466,8 +9466,8 @@
         <v>267</v>
       </c>
     </row>
-    <row r="119" spans="2:33" ht="15" thickBot="1"/>
-    <row r="120" spans="2:33" ht="24" thickBot="1">
+    <row r="119" spans="2:33" ht="14.4" thickBot="1"/>
+    <row r="120" spans="2:33" ht="23.4" thickBot="1">
       <c r="B120" s="10" t="s">
         <v>268</v>
       </c>
@@ -9490,7 +9490,7 @@
       <c r="S120" s="11"/>
       <c r="T120" s="12"/>
     </row>
-    <row r="121" spans="2:33" ht="17.25">
+    <row r="121" spans="2:33" ht="17.399999999999999">
       <c r="B121" s="9" t="s">
         <v>269</v>
       </c>
@@ -9501,7 +9501,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="122" spans="2:33" ht="15">
+    <row r="122" spans="2:33">
       <c r="B122" s="4" t="s">
         <v>272</v>
       </c>
@@ -9561,7 +9561,7 @@
       <c r="R127" s="4"/>
       <c r="AG127" s="4"/>
     </row>
-    <row r="128" spans="2:33" ht="15">
+    <row r="128" spans="2:33">
       <c r="B128" s="4" t="s">
         <v>287</v>
       </c>
@@ -9620,7 +9620,7 @@
       <c r="B133" s="4"/>
       <c r="R133" s="4"/>
     </row>
-    <row r="134" spans="2:33" ht="15">
+    <row r="134" spans="2:33">
       <c r="B134" s="4" t="s">
         <v>302</v>
       </c>
@@ -9663,7 +9663,7 @@
     <row r="139" spans="2:33">
       <c r="B139" s="4"/>
     </row>
-    <row r="140" spans="2:33" ht="15">
+    <row r="140" spans="2:33">
       <c r="B140" s="4" t="s">
         <v>312</v>
       </c>
@@ -9688,7 +9688,7 @@
         <v>316</v>
       </c>
     </row>
-    <row r="146" spans="2:48" ht="23.25">
+    <row r="146" spans="2:48" ht="22.8">
       <c r="B146" s="13" t="s">
         <v>317</v>
       </c>
@@ -9715,7 +9715,7 @@
       <c r="W146" s="14"/>
       <c r="X146" s="14"/>
     </row>
-    <row r="147" spans="2:48" ht="17.25">
+    <row r="147" spans="2:48" ht="17.399999999999999">
       <c r="B147" s="9" t="s">
         <v>318</v>
       </c>
@@ -9729,7 +9729,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="148" spans="2:48" ht="15">
+    <row r="148" spans="2:48">
       <c r="B148" s="4" t="s">
         <v>322</v>
       </c>
@@ -9805,7 +9805,7 @@
       <c r="AG153" s="4"/>
       <c r="AV153" s="4"/>
     </row>
-    <row r="154" spans="2:48" ht="15">
+    <row r="154" spans="2:48">
       <c r="B154" s="4" t="s">
         <v>342</v>
       </c>
@@ -9881,7 +9881,7 @@
       <c r="AG159" s="4"/>
       <c r="AV159" s="4"/>
     </row>
-    <row r="160" spans="2:48" ht="15">
+    <row r="160" spans="2:48">
       <c r="B160" s="4" t="s">
         <v>362</v>
       </c>
@@ -9954,7 +9954,7 @@
     <row r="165" spans="2:48">
       <c r="R165" s="4"/>
     </row>
-    <row r="166" spans="2:48" ht="15">
+    <row r="166" spans="2:48">
       <c r="R166" s="4" t="s">
         <v>382</v>
       </c>
@@ -9979,8 +9979,8 @@
         <v>386</v>
       </c>
     </row>
-    <row r="172" spans="2:48" ht="15" thickBot="1"/>
-    <row r="173" spans="2:48" ht="24" thickBot="1">
+    <row r="172" spans="2:48" ht="14.4" thickBot="1"/>
+    <row r="173" spans="2:48" ht="23.4" thickBot="1">
       <c r="B173" s="10" t="s">
         <v>387</v>
       </c>
@@ -9999,7 +9999,7 @@
       <c r="O173" s="11"/>
       <c r="P173" s="12"/>
     </row>
-    <row r="174" spans="2:48" ht="17.25">
+    <row r="174" spans="2:48" ht="17.399999999999999">
       <c r="B174" s="9" t="s">
         <v>388</v>
       </c>
@@ -10007,7 +10007,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="175" spans="2:48" ht="15">
+    <row r="175" spans="2:48">
       <c r="B175" s="4" t="s">
         <v>390</v>
       </c>
@@ -10051,7 +10051,7 @@
       <c r="B180" s="4"/>
       <c r="R180" s="4"/>
     </row>
-    <row r="181" spans="2:18" ht="15">
+    <row r="181" spans="2:18">
       <c r="B181" s="4" t="s">
         <v>400</v>
       </c>
@@ -10094,7 +10094,7 @@
     <row r="186" spans="2:18">
       <c r="B186" s="4"/>
     </row>
-    <row r="187" spans="2:18" ht="15">
+    <row r="187" spans="2:18">
       <c r="B187" s="4" t="s">
         <v>410</v>
       </c>
@@ -10122,7 +10122,7 @@
     <row r="192" spans="2:18">
       <c r="B192" s="4"/>
     </row>
-    <row r="193" spans="2:29" ht="15">
+    <row r="193" spans="2:29">
       <c r="B193" s="4" t="s">
         <v>415</v>
       </c>
@@ -10147,8 +10147,8 @@
         <v>419</v>
       </c>
     </row>
-    <row r="198" spans="2:29" ht="15" thickBot="1"/>
-    <row r="199" spans="2:29" ht="24" thickBot="1">
+    <row r="198" spans="2:29" ht="14.4" thickBot="1"/>
+    <row r="199" spans="2:29" ht="23.4" thickBot="1">
       <c r="B199" s="10" t="s">
         <v>420</v>
       </c>
@@ -10166,7 +10166,7 @@
       <c r="N199" s="11"/>
       <c r="O199" s="12"/>
     </row>
-    <row r="200" spans="2:29" ht="17.25">
+    <row r="200" spans="2:29" ht="17.399999999999999">
       <c r="B200" s="9" t="s">
         <v>421</v>
       </c>
@@ -10177,7 +10177,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="201" spans="2:29" ht="15">
+    <row r="201" spans="2:29">
       <c r="B201" s="4" t="s">
         <v>424</v>
       </c>
@@ -10237,7 +10237,7 @@
       <c r="R206" s="4"/>
       <c r="AC206" s="4"/>
     </row>
-    <row r="207" spans="2:29" ht="15">
+    <row r="207" spans="2:29">
       <c r="B207" s="4" t="s">
         <v>439</v>
       </c>
@@ -10295,7 +10295,7 @@
     <row r="212" spans="2:33">
       <c r="B212" s="4"/>
     </row>
-    <row r="213" spans="2:33" ht="15">
+    <row r="213" spans="2:33">
       <c r="B213" s="4" t="s">
         <v>454</v>
       </c>
@@ -10320,8 +10320,8 @@
         <v>458</v>
       </c>
     </row>
-    <row r="219" spans="2:33" ht="15" thickBot="1"/>
-    <row r="220" spans="2:33" ht="24" thickBot="1">
+    <row r="219" spans="2:33" ht="14.4" thickBot="1"/>
+    <row r="220" spans="2:33" ht="23.4" thickBot="1">
       <c r="B220" s="10" t="s">
         <v>459</v>
       </c>
@@ -10340,7 +10340,7 @@
       <c r="O220" s="11"/>
       <c r="P220" s="12"/>
     </row>
-    <row r="221" spans="2:33" ht="17.25">
+    <row r="221" spans="2:33" ht="17.399999999999999">
       <c r="B221" s="9" t="s">
         <v>460</v>
       </c>
@@ -10351,7 +10351,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="222" spans="2:33" ht="15">
+    <row r="222" spans="2:33">
       <c r="B222" s="4" t="s">
         <v>463</v>
       </c>
@@ -10411,7 +10411,7 @@
       <c r="P227" s="4"/>
       <c r="AG227" s="4"/>
     </row>
-    <row r="228" spans="2:33" ht="15">
+    <row r="228" spans="2:33">
       <c r="B228" s="4" t="s">
         <v>478</v>
       </c>
@@ -10472,13 +10472,13 @@
       </c>
       <c r="P233" s="4"/>
     </row>
-    <row r="234" spans="2:33" ht="15">
+    <row r="234" spans="2:33">
       <c r="B234" s="4"/>
       <c r="P234" s="4" t="s">
         <v>494</v>
       </c>
     </row>
-    <row r="235" spans="2:33" ht="15">
+    <row r="235" spans="2:33">
       <c r="B235" s="4" t="s">
         <v>495</v>
       </c>
@@ -10515,8 +10515,8 @@
         <v>503</v>
       </c>
     </row>
-    <row r="240" spans="2:33" ht="15" thickBot="1"/>
-    <row r="241" spans="2:33" ht="24" thickBot="1">
+    <row r="240" spans="2:33" ht="14.4" thickBot="1"/>
+    <row r="241" spans="2:33" ht="23.4" thickBot="1">
       <c r="B241" s="10" t="s">
         <v>504</v>
       </c>
@@ -10534,7 +10534,7 @@
       <c r="N241" s="11"/>
       <c r="O241" s="12"/>
     </row>
-    <row r="242" spans="2:33" ht="17.25">
+    <row r="242" spans="2:33" ht="17.399999999999999">
       <c r="B242" s="9" t="s">
         <v>505</v>
       </c>
@@ -10545,7 +10545,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="243" spans="2:33" ht="15">
+    <row r="243" spans="2:33">
       <c r="B243" s="4" t="s">
         <v>508</v>
       </c>
@@ -10605,7 +10605,7 @@
       <c r="P248" s="4"/>
       <c r="AG248" s="4"/>
     </row>
-    <row r="249" spans="2:33" ht="15">
+    <row r="249" spans="2:33">
       <c r="B249" s="4" t="s">
         <v>523</v>
       </c>
@@ -10664,7 +10664,7 @@
       <c r="B254" s="4"/>
       <c r="P254" s="4"/>
     </row>
-    <row r="255" spans="2:33" ht="15">
+    <row r="255" spans="2:33">
       <c r="B255" s="4" t="s">
         <v>538</v>
       </c>
@@ -10704,32 +10704,32 @@
         <v>547</v>
       </c>
     </row>
-    <row r="260" spans="2:41" ht="15" thickBot="1"/>
-    <row r="261" spans="2:41" ht="24" thickBot="1">
-      <c r="B261" s="6" t="s">
+    <row r="260" spans="2:41" ht="14.4" thickBot="1"/>
+    <row r="261" spans="2:41" ht="23.4" thickBot="1">
+      <c r="B261" s="10" t="s">
         <v>548</v>
       </c>
-      <c r="C261" s="7"/>
-      <c r="D261" s="7"/>
-      <c r="E261" s="7"/>
-      <c r="F261" s="7"/>
-      <c r="G261" s="7"/>
-      <c r="H261" s="7"/>
-      <c r="I261" s="7"/>
-      <c r="J261" s="7"/>
-      <c r="K261" s="7"/>
-      <c r="L261" s="7"/>
-      <c r="M261" s="7"/>
-      <c r="N261" s="7"/>
-      <c r="O261" s="7"/>
-      <c r="P261" s="7"/>
-      <c r="Q261" s="7"/>
-      <c r="R261" s="7"/>
-      <c r="S261" s="7"/>
-      <c r="T261" s="7"/>
-      <c r="U261" s="8"/>
-    </row>
-    <row r="262" spans="2:41" ht="17.25">
+      <c r="C261" s="11"/>
+      <c r="D261" s="11"/>
+      <c r="E261" s="11"/>
+      <c r="F261" s="11"/>
+      <c r="G261" s="11"/>
+      <c r="H261" s="11"/>
+      <c r="I261" s="11"/>
+      <c r="J261" s="11"/>
+      <c r="K261" s="11"/>
+      <c r="L261" s="11"/>
+      <c r="M261" s="11"/>
+      <c r="N261" s="11"/>
+      <c r="O261" s="11"/>
+      <c r="P261" s="11"/>
+      <c r="Q261" s="11"/>
+      <c r="R261" s="11"/>
+      <c r="S261" s="11"/>
+      <c r="T261" s="11"/>
+      <c r="U261" s="12"/>
+    </row>
+    <row r="262" spans="2:41" ht="17.399999999999999">
       <c r="B262" s="9" t="s">
         <v>549</v>
       </c>
@@ -10743,7 +10743,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="263" spans="2:41" ht="15">
+    <row r="263" spans="2:41">
       <c r="B263" s="4" t="s">
         <v>553</v>
       </c>
@@ -10821,7 +10821,7 @@
         <v>573</v>
       </c>
     </row>
-    <row r="269" spans="2:41" ht="15">
+    <row r="269" spans="2:41">
       <c r="B269" s="4" t="s">
         <v>574</v>
       </c>
@@ -10833,7 +10833,7 @@
       </c>
       <c r="AO269" s="4"/>
     </row>
-    <row r="270" spans="2:41" ht="15">
+    <row r="270" spans="2:41">
       <c r="B270" s="5" t="s">
         <v>577</v>
       </c>
@@ -10896,7 +10896,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="275" spans="2:41" ht="15">
+    <row r="275" spans="2:41">
       <c r="B275" s="4" t="s">
         <v>594</v>
       </c>
@@ -10941,29 +10941,29 @@
         <v>604</v>
       </c>
     </row>
-    <row r="281" spans="2:41" ht="15" thickBot="1"/>
-    <row r="282" spans="2:41" ht="24" thickBot="1">
-      <c r="B282" s="6" t="s">
+    <row r="281" spans="2:41" ht="14.4" thickBot="1"/>
+    <row r="282" spans="2:41" ht="23.4" thickBot="1">
+      <c r="B282" s="10" t="s">
         <v>605</v>
       </c>
-      <c r="C282" s="7"/>
-      <c r="D282" s="7"/>
-      <c r="E282" s="7"/>
-      <c r="F282" s="7"/>
-      <c r="G282" s="7"/>
-      <c r="H282" s="7"/>
-      <c r="I282" s="7"/>
-      <c r="J282" s="7"/>
-      <c r="K282" s="7"/>
-      <c r="L282" s="7"/>
-      <c r="M282" s="7"/>
-      <c r="N282" s="7"/>
-      <c r="O282" s="7"/>
-      <c r="P282" s="7"/>
-      <c r="Q282" s="7"/>
-      <c r="R282" s="8"/>
-    </row>
-    <row r="283" spans="2:41" ht="17.25">
+      <c r="C282" s="11"/>
+      <c r="D282" s="11"/>
+      <c r="E282" s="11"/>
+      <c r="F282" s="11"/>
+      <c r="G282" s="11"/>
+      <c r="H282" s="11"/>
+      <c r="I282" s="11"/>
+      <c r="J282" s="11"/>
+      <c r="K282" s="11"/>
+      <c r="L282" s="11"/>
+      <c r="M282" s="11"/>
+      <c r="N282" s="11"/>
+      <c r="O282" s="11"/>
+      <c r="P282" s="11"/>
+      <c r="Q282" s="11"/>
+      <c r="R282" s="12"/>
+    </row>
+    <row r="283" spans="2:41" ht="17.399999999999999">
       <c r="B283" s="9" t="s">
         <v>606</v>
       </c>
@@ -10974,7 +10974,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="284" spans="2:41" ht="15">
+    <row r="284" spans="2:41">
       <c r="B284" s="4" t="s">
         <v>609</v>
       </c>
@@ -11034,7 +11034,7 @@
       <c r="Q289" s="4"/>
       <c r="AC289" s="4"/>
     </row>
-    <row r="290" spans="2:29" ht="15">
+    <row r="290" spans="2:29">
       <c r="B290" s="4" t="s">
         <v>624</v>
       </c>
@@ -11092,7 +11092,7 @@
     <row r="295" spans="2:29">
       <c r="B295" s="4"/>
     </row>
-    <row r="296" spans="2:29" ht="15">
+    <row r="296" spans="2:29">
       <c r="B296" s="4" t="s">
         <v>639</v>
       </c>
@@ -11117,33 +11117,33 @@
         <v>642</v>
       </c>
     </row>
-    <row r="301" spans="2:29" ht="15" thickBot="1"/>
-    <row r="302" spans="2:29" ht="24" thickBot="1">
-      <c r="B302" s="6" t="s">
+    <row r="301" spans="2:29" ht="14.4" thickBot="1"/>
+    <row r="302" spans="2:29" ht="23.4" thickBot="1">
+      <c r="B302" s="10" t="s">
         <v>643</v>
       </c>
-      <c r="C302" s="7"/>
-      <c r="D302" s="7"/>
-      <c r="E302" s="7"/>
-      <c r="F302" s="7"/>
-      <c r="G302" s="7"/>
-      <c r="H302" s="7"/>
-      <c r="I302" s="7"/>
-      <c r="J302" s="7"/>
-      <c r="K302" s="7"/>
-      <c r="L302" s="7"/>
-      <c r="M302" s="7"/>
-      <c r="N302" s="7"/>
-      <c r="O302" s="7"/>
-      <c r="P302" s="7"/>
-      <c r="Q302" s="7"/>
-      <c r="R302" s="7"/>
-      <c r="S302" s="7"/>
-      <c r="T302" s="7"/>
-      <c r="U302" s="7"/>
-      <c r="V302" s="8"/>
-    </row>
-    <row r="303" spans="2:29" ht="17.25">
+      <c r="C302" s="11"/>
+      <c r="D302" s="11"/>
+      <c r="E302" s="11"/>
+      <c r="F302" s="11"/>
+      <c r="G302" s="11"/>
+      <c r="H302" s="11"/>
+      <c r="I302" s="11"/>
+      <c r="J302" s="11"/>
+      <c r="K302" s="11"/>
+      <c r="L302" s="11"/>
+      <c r="M302" s="11"/>
+      <c r="N302" s="11"/>
+      <c r="O302" s="11"/>
+      <c r="P302" s="11"/>
+      <c r="Q302" s="11"/>
+      <c r="R302" s="11"/>
+      <c r="S302" s="11"/>
+      <c r="T302" s="11"/>
+      <c r="U302" s="11"/>
+      <c r="V302" s="12"/>
+    </row>
+    <row r="303" spans="2:29" ht="17.399999999999999">
       <c r="B303" s="9" t="s">
         <v>644</v>
       </c>
@@ -11154,7 +11154,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="304" spans="2:29" ht="15">
+    <row r="304" spans="2:29">
       <c r="B304" s="4" t="s">
         <v>647</v>
       </c>
@@ -11214,7 +11214,7 @@
       <c r="P309" s="4"/>
       <c r="AC309" s="4"/>
     </row>
-    <row r="310" spans="2:29" ht="15">
+    <row r="310" spans="2:29">
       <c r="B310" s="4" t="s">
         <v>662</v>
       </c>
@@ -11269,30 +11269,30 @@
         <v>676</v>
       </c>
     </row>
-    <row r="315" spans="2:29" ht="15" thickBot="1"/>
-    <row r="316" spans="2:29" ht="24" thickBot="1">
-      <c r="B316" s="6" t="s">
+    <row r="315" spans="2:29" ht="14.4" thickBot="1"/>
+    <row r="316" spans="2:29" ht="23.4" thickBot="1">
+      <c r="B316" s="10" t="s">
         <v>677</v>
       </c>
-      <c r="C316" s="7"/>
-      <c r="D316" s="7"/>
-      <c r="E316" s="7"/>
-      <c r="F316" s="7"/>
-      <c r="G316" s="7"/>
-      <c r="H316" s="7"/>
-      <c r="I316" s="7"/>
-      <c r="J316" s="7"/>
-      <c r="K316" s="7"/>
-      <c r="L316" s="7"/>
-      <c r="M316" s="7"/>
-      <c r="N316" s="7"/>
-      <c r="O316" s="7"/>
-      <c r="P316" s="7"/>
-      <c r="Q316" s="7"/>
-      <c r="R316" s="7"/>
-      <c r="S316" s="8"/>
-    </row>
-    <row r="317" spans="2:29" ht="17.25">
+      <c r="C316" s="11"/>
+      <c r="D316" s="11"/>
+      <c r="E316" s="11"/>
+      <c r="F316" s="11"/>
+      <c r="G316" s="11"/>
+      <c r="H316" s="11"/>
+      <c r="I316" s="11"/>
+      <c r="J316" s="11"/>
+      <c r="K316" s="11"/>
+      <c r="L316" s="11"/>
+      <c r="M316" s="11"/>
+      <c r="N316" s="11"/>
+      <c r="O316" s="11"/>
+      <c r="P316" s="11"/>
+      <c r="Q316" s="11"/>
+      <c r="R316" s="11"/>
+      <c r="S316" s="12"/>
+    </row>
+    <row r="317" spans="2:29" ht="17.399999999999999">
       <c r="B317" s="9" t="s">
         <v>678</v>
       </c>
@@ -11303,7 +11303,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="318" spans="2:29" ht="15">
+    <row r="318" spans="2:29">
       <c r="B318" s="4" t="s">
         <v>681</v>
       </c>
@@ -11362,7 +11362,7 @@
       <c r="B323" s="4"/>
       <c r="P323" s="4"/>
     </row>
-    <row r="324" spans="2:52" ht="15">
+    <row r="324" spans="2:52">
       <c r="B324" s="4" t="s">
         <v>695</v>
       </c>
@@ -11402,25 +11402,25 @@
         <v>704</v>
       </c>
     </row>
-    <row r="329" spans="2:52" ht="15" thickBot="1"/>
-    <row r="330" spans="2:52" ht="24" thickBot="1">
-      <c r="B330" s="6" t="s">
+    <row r="329" spans="2:52" ht="14.4" thickBot="1"/>
+    <row r="330" spans="2:52" ht="23.4" thickBot="1">
+      <c r="B330" s="10" t="s">
         <v>705</v>
       </c>
-      <c r="C330" s="7"/>
-      <c r="D330" s="7"/>
-      <c r="E330" s="7"/>
-      <c r="F330" s="7"/>
-      <c r="G330" s="7"/>
-      <c r="H330" s="7"/>
-      <c r="I330" s="7"/>
-      <c r="J330" s="7"/>
-      <c r="K330" s="7"/>
-      <c r="L330" s="7"/>
-      <c r="M330" s="7"/>
-      <c r="N330" s="8"/>
-    </row>
-    <row r="331" spans="2:52" ht="17.25">
+      <c r="C330" s="11"/>
+      <c r="D330" s="11"/>
+      <c r="E330" s="11"/>
+      <c r="F330" s="11"/>
+      <c r="G330" s="11"/>
+      <c r="H330" s="11"/>
+      <c r="I330" s="11"/>
+      <c r="J330" s="11"/>
+      <c r="K330" s="11"/>
+      <c r="L330" s="11"/>
+      <c r="M330" s="11"/>
+      <c r="N330" s="12"/>
+    </row>
+    <row r="331" spans="2:52" ht="17.399999999999999">
       <c r="B331" s="9" t="s">
         <v>706</v>
       </c>
@@ -11522,8 +11522,8 @@
         <v>735</v>
       </c>
     </row>
-    <row r="337" spans="2:29" ht="15" thickBot="1"/>
-    <row r="338" spans="2:29" ht="24" thickBot="1">
+    <row r="337" spans="2:29" ht="14.4" thickBot="1"/>
+    <row r="338" spans="2:29" ht="23.4" thickBot="1">
       <c r="B338" s="6" t="s">
         <v>736</v>
       </c>
@@ -11541,7 +11541,7 @@
       <c r="N338" s="7"/>
       <c r="O338" s="8"/>
     </row>
-    <row r="339" spans="2:29" ht="17.25">
+    <row r="339" spans="2:29" ht="17.399999999999999">
       <c r="B339" s="9" t="s">
         <v>737</v>
       </c>
@@ -11552,7 +11552,7 @@
         <v>739</v>
       </c>
     </row>
-    <row r="340" spans="2:29" ht="15">
+    <row r="340" spans="2:29">
       <c r="B340" s="4" t="s">
         <v>740</v>
       </c>
@@ -11612,7 +11612,7 @@
       <c r="P345" s="4"/>
       <c r="AC345" s="4"/>
     </row>
-    <row r="346" spans="2:29" ht="15">
+    <row r="346" spans="2:29">
       <c r="B346" s="4" t="s">
         <v>755</v>
       </c>

</xml_diff>